<commit_message>
Update Excel file via delegated auth - Tue Oct 13 15:36:27 UTC 2026
</commit_message>
<xml_diff>
--- a/data/Recognitions_latest.xlsx
+++ b/data/Recognitions_latest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aphrcorg-my.sharepoint.com/personal/nnjenga_aphrc_org/Documents/CARTA Dashboard/ECRS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="746" documentId="13_ncr:1_{74C5384D-9D49-4106-BD43-FCAED859190D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4810BA06-6DCB-4B0B-9070-65E5FDBD30E7}"/>
+  <xr:revisionPtr revIDLastSave="755" documentId="13_ncr:1_{74C5384D-9D49-4106-BD43-FCAED859190D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6997F9E1-9AD9-4AB1-94B5-D0D96AB3A1B2}"/>
   <bookViews>
     <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,10 +24,10 @@
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="330" r:id="rId6"/>
-    <pivotCache cacheId="331" r:id="rId7"/>
-    <pivotCache cacheId="332" r:id="rId8"/>
-    <pivotCache cacheId="333" r:id="rId9"/>
+    <pivotCache cacheId="471" r:id="rId6"/>
+    <pivotCache cacheId="472" r:id="rId7"/>
+    <pivotCache cacheId="473" r:id="rId8"/>
+    <pivotCache cacheId="474" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -121,7 +121,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3080" uniqueCount="808">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3088" uniqueCount="809">
   <si>
     <t>No</t>
   </si>
@@ -2520,6 +2520,9 @@
   </si>
   <si>
     <t>Appointed Extraordinary Research Fellow at the Africa Center for Inclusive Health Management at Stellenbosch University, South Africa, from July 1, 2026, to June 30, 2029. I</t>
+  </si>
+  <si>
+    <t>Appointed Director, Ifakara Health Institute</t>
   </si>
   <si>
     <t>(All)</t>
@@ -26972,106 +26975,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{55E369D5-46AA-45F8-B4A0-AC6C0CED6464}" name="PivotTable2" cacheId="330" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="A3:D9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="16">
-    <pivotField dataField="1" compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField axis="axisCol" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item m="1" x="2"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="5">
-        <item x="0"/>
-        <item m="1" x="4"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="1"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" defaultSubtotal="0">
-      <items count="9">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="1"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="4"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="3"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <pageFields count="1">
-    <pageField fld="8" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Count of No" fld="0" subtotal="count" baseField="4" baseItem="3"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{414D3242-6D58-4EC3-BE1F-E4596803BECC}" name="PivotTable10" cacheId="330" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{414D3242-6D58-4EC3-BE1F-E4596803BECC}" name="PivotTable10" cacheId="471" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A16:H19" firstHeaderRow="1" firstDataRow="3" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="16">
     <pivotField dataField="1" compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
@@ -27213,8 +27117,815 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{55E369D5-46AA-45F8-B4A0-AC6C0CED6464}" name="PivotTable2" cacheId="471" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A3:D9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="16">
+    <pivotField dataField="1" compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField axis="axisCol" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item m="1" x="2"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="5">
+        <item x="0"/>
+        <item m="1" x="4"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="1"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField axis="axisPage" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" defaultSubtotal="0">
+      <items count="9">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="1"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+    <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="3"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="8" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Count of No" fld="0" subtotal="count" baseField="4" baseItem="3"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C759C715-A218-40D6-B8AD-8DD0CC6815DF}" name="PivotTable1" cacheId="333" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{90770DB3-F829-4E9E-88FA-FB5C22EB6463}" name="PivotTable2" cacheId="473" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="D4:E146" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
+  <pivotFields count="18">
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="142">
+        <item x="57"/>
+        <item x="116"/>
+        <item x="10"/>
+        <item x="27"/>
+        <item x="88"/>
+        <item x="19"/>
+        <item x="14"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="125"/>
+        <item x="128"/>
+        <item x="121"/>
+        <item x="41"/>
+        <item x="80"/>
+        <item x="93"/>
+        <item x="81"/>
+        <item x="111"/>
+        <item x="82"/>
+        <item x="49"/>
+        <item x="48"/>
+        <item x="68"/>
+        <item x="107"/>
+        <item x="83"/>
+        <item x="42"/>
+        <item x="97"/>
+        <item x="5"/>
+        <item x="11"/>
+        <item x="8"/>
+        <item x="35"/>
+        <item x="25"/>
+        <item x="99"/>
+        <item x="32"/>
+        <item x="22"/>
+        <item x="9"/>
+        <item x="13"/>
+        <item x="126"/>
+        <item x="54"/>
+        <item x="28"/>
+        <item x="53"/>
+        <item x="21"/>
+        <item x="84"/>
+        <item x="20"/>
+        <item x="12"/>
+        <item x="1"/>
+        <item x="86"/>
+        <item x="102"/>
+        <item x="127"/>
+        <item x="30"/>
+        <item x="43"/>
+        <item x="85"/>
+        <item x="112"/>
+        <item x="62"/>
+        <item x="50"/>
+        <item x="98"/>
+        <item x="36"/>
+        <item x="106"/>
+        <item x="17"/>
+        <item x="6"/>
+        <item x="122"/>
+        <item x="52"/>
+        <item x="104"/>
+        <item x="3"/>
+        <item x="7"/>
+        <item x="18"/>
+        <item x="26"/>
+        <item x="103"/>
+        <item x="31"/>
+        <item x="89"/>
+        <item x="118"/>
+        <item x="2"/>
+        <item x="16"/>
+        <item x="55"/>
+        <item x="58"/>
+        <item x="114"/>
+        <item x="33"/>
+        <item x="87"/>
+        <item x="113"/>
+        <item x="69"/>
+        <item x="51"/>
+        <item x="59"/>
+        <item x="101"/>
+        <item x="34"/>
+        <item x="109"/>
+        <item x="61"/>
+        <item x="132"/>
+        <item x="56"/>
+        <item x="64"/>
+        <item x="117"/>
+        <item x="63"/>
+        <item x="100"/>
+        <item x="124"/>
+        <item x="108"/>
+        <item x="115"/>
+        <item x="70"/>
+        <item x="71"/>
+        <item x="72"/>
+        <item x="4"/>
+        <item x="15"/>
+        <item x="65"/>
+        <item x="44"/>
+        <item x="119"/>
+        <item x="105"/>
+        <item x="66"/>
+        <item x="120"/>
+        <item x="123"/>
+        <item x="45"/>
+        <item x="129"/>
+        <item x="130"/>
+        <item x="39"/>
+        <item x="73"/>
+        <item x="110"/>
+        <item x="46"/>
+        <item x="94"/>
+        <item x="74"/>
+        <item x="29"/>
+        <item x="75"/>
+        <item x="90"/>
+        <item x="67"/>
+        <item x="76"/>
+        <item x="38"/>
+        <item x="91"/>
+        <item x="37"/>
+        <item x="40"/>
+        <item x="60"/>
+        <item x="95"/>
+        <item x="77"/>
+        <item x="47"/>
+        <item x="78"/>
+        <item x="131"/>
+        <item x="96"/>
+        <item x="92"/>
+        <item x="79"/>
+        <item x="0"/>
+        <item x="133"/>
+        <item x="134"/>
+        <item x="135"/>
+        <item x="136"/>
+        <item x="137"/>
+        <item x="138"/>
+        <item x="139"/>
+        <item x="140"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisPage" compact="0" outline="0" showAll="0">
+      <items count="12">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="1"/>
+        <item x="10"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisPage" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="69">
+        <item x="57"/>
+        <item x="56"/>
+        <item x="55"/>
+        <item x="39"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="43"/>
+        <item x="20"/>
+        <item x="35"/>
+        <item x="46"/>
+        <item x="47"/>
+        <item x="50"/>
+        <item x="23"/>
+        <item x="16"/>
+        <item x="52"/>
+        <item x="30"/>
+        <item x="12"/>
+        <item x="24"/>
+        <item x="63"/>
+        <item x="31"/>
+        <item x="17"/>
+        <item x="28"/>
+        <item x="37"/>
+        <item x="48"/>
+        <item x="13"/>
+        <item x="32"/>
+        <item x="51"/>
+        <item x="22"/>
+        <item x="36"/>
+        <item x="54"/>
+        <item x="49"/>
+        <item x="18"/>
+        <item x="53"/>
+        <item x="19"/>
+        <item x="26"/>
+        <item x="45"/>
+        <item x="64"/>
+        <item x="42"/>
+        <item x="62"/>
+        <item x="29"/>
+        <item x="38"/>
+        <item x="15"/>
+        <item x="33"/>
+        <item x="34"/>
+        <item x="44"/>
+        <item x="21"/>
+        <item x="25"/>
+        <item x="27"/>
+        <item x="41"/>
+        <item x="61"/>
+        <item x="58"/>
+        <item x="60"/>
+        <item x="6"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="11"/>
+        <item x="10"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="40"/>
+        <item x="1"/>
+        <item x="14"/>
+        <item x="59"/>
+        <item x="0"/>
+        <item x="65"/>
+        <item x="66"/>
+        <item x="67"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="142">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="20"/>
+    </i>
+    <i>
+      <x v="21"/>
+    </i>
+    <i>
+      <x v="22"/>
+    </i>
+    <i>
+      <x v="23"/>
+    </i>
+    <i>
+      <x v="24"/>
+    </i>
+    <i>
+      <x v="25"/>
+    </i>
+    <i>
+      <x v="26"/>
+    </i>
+    <i>
+      <x v="27"/>
+    </i>
+    <i>
+      <x v="28"/>
+    </i>
+    <i>
+      <x v="29"/>
+    </i>
+    <i>
+      <x v="30"/>
+    </i>
+    <i>
+      <x v="31"/>
+    </i>
+    <i>
+      <x v="32"/>
+    </i>
+    <i>
+      <x v="33"/>
+    </i>
+    <i>
+      <x v="34"/>
+    </i>
+    <i>
+      <x v="35"/>
+    </i>
+    <i>
+      <x v="36"/>
+    </i>
+    <i>
+      <x v="37"/>
+    </i>
+    <i>
+      <x v="38"/>
+    </i>
+    <i>
+      <x v="39"/>
+    </i>
+    <i>
+      <x v="40"/>
+    </i>
+    <i>
+      <x v="41"/>
+    </i>
+    <i>
+      <x v="42"/>
+    </i>
+    <i>
+      <x v="43"/>
+    </i>
+    <i>
+      <x v="44"/>
+    </i>
+    <i>
+      <x v="45"/>
+    </i>
+    <i>
+      <x v="46"/>
+    </i>
+    <i>
+      <x v="47"/>
+    </i>
+    <i>
+      <x v="48"/>
+    </i>
+    <i>
+      <x v="49"/>
+    </i>
+    <i>
+      <x v="50"/>
+    </i>
+    <i>
+      <x v="51"/>
+    </i>
+    <i>
+      <x v="52"/>
+    </i>
+    <i>
+      <x v="53"/>
+    </i>
+    <i>
+      <x v="54"/>
+    </i>
+    <i>
+      <x v="55"/>
+    </i>
+    <i>
+      <x v="56"/>
+    </i>
+    <i>
+      <x v="57"/>
+    </i>
+    <i>
+      <x v="58"/>
+    </i>
+    <i>
+      <x v="59"/>
+    </i>
+    <i>
+      <x v="60"/>
+    </i>
+    <i>
+      <x v="61"/>
+    </i>
+    <i>
+      <x v="62"/>
+    </i>
+    <i>
+      <x v="63"/>
+    </i>
+    <i>
+      <x v="64"/>
+    </i>
+    <i>
+      <x v="65"/>
+    </i>
+    <i>
+      <x v="66"/>
+    </i>
+    <i>
+      <x v="67"/>
+    </i>
+    <i>
+      <x v="68"/>
+    </i>
+    <i>
+      <x v="69"/>
+    </i>
+    <i>
+      <x v="70"/>
+    </i>
+    <i>
+      <x v="71"/>
+    </i>
+    <i>
+      <x v="72"/>
+    </i>
+    <i>
+      <x v="73"/>
+    </i>
+    <i>
+      <x v="74"/>
+    </i>
+    <i>
+      <x v="75"/>
+    </i>
+    <i>
+      <x v="76"/>
+    </i>
+    <i>
+      <x v="77"/>
+    </i>
+    <i>
+      <x v="78"/>
+    </i>
+    <i>
+      <x v="79"/>
+    </i>
+    <i>
+      <x v="80"/>
+    </i>
+    <i>
+      <x v="81"/>
+    </i>
+    <i>
+      <x v="82"/>
+    </i>
+    <i>
+      <x v="83"/>
+    </i>
+    <i>
+      <x v="84"/>
+    </i>
+    <i>
+      <x v="85"/>
+    </i>
+    <i>
+      <x v="86"/>
+    </i>
+    <i>
+      <x v="87"/>
+    </i>
+    <i>
+      <x v="88"/>
+    </i>
+    <i>
+      <x v="89"/>
+    </i>
+    <i>
+      <x v="90"/>
+    </i>
+    <i>
+      <x v="91"/>
+    </i>
+    <i>
+      <x v="92"/>
+    </i>
+    <i>
+      <x v="93"/>
+    </i>
+    <i>
+      <x v="94"/>
+    </i>
+    <i>
+      <x v="95"/>
+    </i>
+    <i>
+      <x v="96"/>
+    </i>
+    <i>
+      <x v="97"/>
+    </i>
+    <i>
+      <x v="98"/>
+    </i>
+    <i>
+      <x v="99"/>
+    </i>
+    <i>
+      <x v="100"/>
+    </i>
+    <i>
+      <x v="101"/>
+    </i>
+    <i>
+      <x v="102"/>
+    </i>
+    <i>
+      <x v="103"/>
+    </i>
+    <i>
+      <x v="104"/>
+    </i>
+    <i>
+      <x v="105"/>
+    </i>
+    <i>
+      <x v="106"/>
+    </i>
+    <i>
+      <x v="107"/>
+    </i>
+    <i>
+      <x v="108"/>
+    </i>
+    <i>
+      <x v="109"/>
+    </i>
+    <i>
+      <x v="110"/>
+    </i>
+    <i>
+      <x v="111"/>
+    </i>
+    <i>
+      <x v="112"/>
+    </i>
+    <i>
+      <x v="113"/>
+    </i>
+    <i>
+      <x v="114"/>
+    </i>
+    <i>
+      <x v="115"/>
+    </i>
+    <i>
+      <x v="116"/>
+    </i>
+    <i>
+      <x v="117"/>
+    </i>
+    <i>
+      <x v="118"/>
+    </i>
+    <i>
+      <x v="119"/>
+    </i>
+    <i>
+      <x v="120"/>
+    </i>
+    <i>
+      <x v="121"/>
+    </i>
+    <i>
+      <x v="122"/>
+    </i>
+    <i>
+      <x v="123"/>
+    </i>
+    <i>
+      <x v="124"/>
+    </i>
+    <i>
+      <x v="125"/>
+    </i>
+    <i>
+      <x v="126"/>
+    </i>
+    <i>
+      <x v="127"/>
+    </i>
+    <i>
+      <x v="128"/>
+    </i>
+    <i>
+      <x v="129"/>
+    </i>
+    <i>
+      <x v="130"/>
+    </i>
+    <i>
+      <x v="131"/>
+    </i>
+    <i>
+      <x v="132"/>
+    </i>
+    <i>
+      <x v="133"/>
+    </i>
+    <i>
+      <x v="134"/>
+    </i>
+    <i>
+      <x v="135"/>
+    </i>
+    <i>
+      <x v="136"/>
+    </i>
+    <i>
+      <x v="137"/>
+    </i>
+    <i>
+      <x v="138"/>
+    </i>
+    <i>
+      <x v="139"/>
+    </i>
+    <i>
+      <x v="140"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="2">
+    <pageField fld="11" hier="-1"/>
+    <pageField fld="9" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Count of Promotion" fld="11" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C759C715-A218-40D6-B8AD-8DD0CC6815DF}" name="PivotTable1" cacheId="474" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A4:B146" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="18">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -27996,1021 +28707,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{90770DB3-F829-4E9E-88FA-FB5C22EB6463}" name="PivotTable2" cacheId="332" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="D4:E146" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
-  <pivotFields count="18">
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
-      <items count="142">
-        <item x="57"/>
-        <item x="116"/>
-        <item x="10"/>
-        <item x="27"/>
-        <item x="88"/>
-        <item x="19"/>
-        <item x="14"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item x="125"/>
-        <item x="128"/>
-        <item x="121"/>
-        <item x="41"/>
-        <item x="80"/>
-        <item x="93"/>
-        <item x="81"/>
-        <item x="111"/>
-        <item x="82"/>
-        <item x="49"/>
-        <item x="48"/>
-        <item x="68"/>
-        <item x="107"/>
-        <item x="83"/>
-        <item x="42"/>
-        <item x="97"/>
-        <item x="5"/>
-        <item x="11"/>
-        <item x="8"/>
-        <item x="35"/>
-        <item x="25"/>
-        <item x="99"/>
-        <item x="32"/>
-        <item x="22"/>
-        <item x="9"/>
-        <item x="13"/>
-        <item x="126"/>
-        <item x="54"/>
-        <item x="28"/>
-        <item x="53"/>
-        <item x="21"/>
-        <item x="84"/>
-        <item x="20"/>
-        <item x="12"/>
-        <item x="1"/>
-        <item x="86"/>
-        <item x="102"/>
-        <item x="127"/>
-        <item x="30"/>
-        <item x="43"/>
-        <item x="85"/>
-        <item x="112"/>
-        <item x="62"/>
-        <item x="50"/>
-        <item x="98"/>
-        <item x="36"/>
-        <item x="106"/>
-        <item x="17"/>
-        <item x="6"/>
-        <item x="122"/>
-        <item x="52"/>
-        <item x="104"/>
-        <item x="3"/>
-        <item x="7"/>
-        <item x="18"/>
-        <item x="26"/>
-        <item x="103"/>
-        <item x="31"/>
-        <item x="89"/>
-        <item x="118"/>
-        <item x="2"/>
-        <item x="16"/>
-        <item x="55"/>
-        <item x="58"/>
-        <item x="114"/>
-        <item x="33"/>
-        <item x="87"/>
-        <item x="113"/>
-        <item x="69"/>
-        <item x="51"/>
-        <item x="59"/>
-        <item x="101"/>
-        <item x="34"/>
-        <item x="109"/>
-        <item x="61"/>
-        <item x="132"/>
-        <item x="56"/>
-        <item x="64"/>
-        <item x="117"/>
-        <item x="63"/>
-        <item x="100"/>
-        <item x="124"/>
-        <item x="108"/>
-        <item x="115"/>
-        <item x="70"/>
-        <item x="71"/>
-        <item x="72"/>
-        <item x="4"/>
-        <item x="15"/>
-        <item x="65"/>
-        <item x="44"/>
-        <item x="119"/>
-        <item x="105"/>
-        <item x="66"/>
-        <item x="120"/>
-        <item x="123"/>
-        <item x="45"/>
-        <item x="129"/>
-        <item x="130"/>
-        <item x="39"/>
-        <item x="73"/>
-        <item x="110"/>
-        <item x="46"/>
-        <item x="94"/>
-        <item x="74"/>
-        <item x="29"/>
-        <item x="75"/>
-        <item x="90"/>
-        <item x="67"/>
-        <item x="76"/>
-        <item x="38"/>
-        <item x="91"/>
-        <item x="37"/>
-        <item x="40"/>
-        <item x="60"/>
-        <item x="95"/>
-        <item x="77"/>
-        <item x="47"/>
-        <item x="78"/>
-        <item x="131"/>
-        <item x="96"/>
-        <item x="92"/>
-        <item x="79"/>
-        <item x="0"/>
-        <item x="133"/>
-        <item x="134"/>
-        <item x="135"/>
-        <item x="136"/>
-        <item x="137"/>
-        <item x="138"/>
-        <item x="139"/>
-        <item x="140"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisPage" compact="0" outline="0" showAll="0">
-      <items count="12">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="1"/>
-        <item x="10"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisPage" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="69">
-        <item x="57"/>
-        <item x="56"/>
-        <item x="55"/>
-        <item x="39"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="43"/>
-        <item x="20"/>
-        <item x="35"/>
-        <item x="46"/>
-        <item x="47"/>
-        <item x="50"/>
-        <item x="23"/>
-        <item x="16"/>
-        <item x="52"/>
-        <item x="30"/>
-        <item x="12"/>
-        <item x="24"/>
-        <item x="63"/>
-        <item x="31"/>
-        <item x="17"/>
-        <item x="28"/>
-        <item x="37"/>
-        <item x="48"/>
-        <item x="13"/>
-        <item x="32"/>
-        <item x="51"/>
-        <item x="22"/>
-        <item x="36"/>
-        <item x="54"/>
-        <item x="49"/>
-        <item x="18"/>
-        <item x="53"/>
-        <item x="19"/>
-        <item x="26"/>
-        <item x="45"/>
-        <item x="64"/>
-        <item x="42"/>
-        <item x="62"/>
-        <item x="29"/>
-        <item x="38"/>
-        <item x="15"/>
-        <item x="33"/>
-        <item x="34"/>
-        <item x="44"/>
-        <item x="21"/>
-        <item x="25"/>
-        <item x="27"/>
-        <item x="41"/>
-        <item x="61"/>
-        <item x="58"/>
-        <item x="60"/>
-        <item x="6"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="11"/>
-        <item x="10"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="40"/>
-        <item x="1"/>
-        <item x="14"/>
-        <item x="59"/>
-        <item x="0"/>
-        <item x="65"/>
-        <item x="66"/>
-        <item x="67"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="142">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="14"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i>
-      <x v="18"/>
-    </i>
-    <i>
-      <x v="19"/>
-    </i>
-    <i>
-      <x v="20"/>
-    </i>
-    <i>
-      <x v="21"/>
-    </i>
-    <i>
-      <x v="22"/>
-    </i>
-    <i>
-      <x v="23"/>
-    </i>
-    <i>
-      <x v="24"/>
-    </i>
-    <i>
-      <x v="25"/>
-    </i>
-    <i>
-      <x v="26"/>
-    </i>
-    <i>
-      <x v="27"/>
-    </i>
-    <i>
-      <x v="28"/>
-    </i>
-    <i>
-      <x v="29"/>
-    </i>
-    <i>
-      <x v="30"/>
-    </i>
-    <i>
-      <x v="31"/>
-    </i>
-    <i>
-      <x v="32"/>
-    </i>
-    <i>
-      <x v="33"/>
-    </i>
-    <i>
-      <x v="34"/>
-    </i>
-    <i>
-      <x v="35"/>
-    </i>
-    <i>
-      <x v="36"/>
-    </i>
-    <i>
-      <x v="37"/>
-    </i>
-    <i>
-      <x v="38"/>
-    </i>
-    <i>
-      <x v="39"/>
-    </i>
-    <i>
-      <x v="40"/>
-    </i>
-    <i>
-      <x v="41"/>
-    </i>
-    <i>
-      <x v="42"/>
-    </i>
-    <i>
-      <x v="43"/>
-    </i>
-    <i>
-      <x v="44"/>
-    </i>
-    <i>
-      <x v="45"/>
-    </i>
-    <i>
-      <x v="46"/>
-    </i>
-    <i>
-      <x v="47"/>
-    </i>
-    <i>
-      <x v="48"/>
-    </i>
-    <i>
-      <x v="49"/>
-    </i>
-    <i>
-      <x v="50"/>
-    </i>
-    <i>
-      <x v="51"/>
-    </i>
-    <i>
-      <x v="52"/>
-    </i>
-    <i>
-      <x v="53"/>
-    </i>
-    <i>
-      <x v="54"/>
-    </i>
-    <i>
-      <x v="55"/>
-    </i>
-    <i>
-      <x v="56"/>
-    </i>
-    <i>
-      <x v="57"/>
-    </i>
-    <i>
-      <x v="58"/>
-    </i>
-    <i>
-      <x v="59"/>
-    </i>
-    <i>
-      <x v="60"/>
-    </i>
-    <i>
-      <x v="61"/>
-    </i>
-    <i>
-      <x v="62"/>
-    </i>
-    <i>
-      <x v="63"/>
-    </i>
-    <i>
-      <x v="64"/>
-    </i>
-    <i>
-      <x v="65"/>
-    </i>
-    <i>
-      <x v="66"/>
-    </i>
-    <i>
-      <x v="67"/>
-    </i>
-    <i>
-      <x v="68"/>
-    </i>
-    <i>
-      <x v="69"/>
-    </i>
-    <i>
-      <x v="70"/>
-    </i>
-    <i>
-      <x v="71"/>
-    </i>
-    <i>
-      <x v="72"/>
-    </i>
-    <i>
-      <x v="73"/>
-    </i>
-    <i>
-      <x v="74"/>
-    </i>
-    <i>
-      <x v="75"/>
-    </i>
-    <i>
-      <x v="76"/>
-    </i>
-    <i>
-      <x v="77"/>
-    </i>
-    <i>
-      <x v="78"/>
-    </i>
-    <i>
-      <x v="79"/>
-    </i>
-    <i>
-      <x v="80"/>
-    </i>
-    <i>
-      <x v="81"/>
-    </i>
-    <i>
-      <x v="82"/>
-    </i>
-    <i>
-      <x v="83"/>
-    </i>
-    <i>
-      <x v="84"/>
-    </i>
-    <i>
-      <x v="85"/>
-    </i>
-    <i>
-      <x v="86"/>
-    </i>
-    <i>
-      <x v="87"/>
-    </i>
-    <i>
-      <x v="88"/>
-    </i>
-    <i>
-      <x v="89"/>
-    </i>
-    <i>
-      <x v="90"/>
-    </i>
-    <i>
-      <x v="91"/>
-    </i>
-    <i>
-      <x v="92"/>
-    </i>
-    <i>
-      <x v="93"/>
-    </i>
-    <i>
-      <x v="94"/>
-    </i>
-    <i>
-      <x v="95"/>
-    </i>
-    <i>
-      <x v="96"/>
-    </i>
-    <i>
-      <x v="97"/>
-    </i>
-    <i>
-      <x v="98"/>
-    </i>
-    <i>
-      <x v="99"/>
-    </i>
-    <i>
-      <x v="100"/>
-    </i>
-    <i>
-      <x v="101"/>
-    </i>
-    <i>
-      <x v="102"/>
-    </i>
-    <i>
-      <x v="103"/>
-    </i>
-    <i>
-      <x v="104"/>
-    </i>
-    <i>
-      <x v="105"/>
-    </i>
-    <i>
-      <x v="106"/>
-    </i>
-    <i>
-      <x v="107"/>
-    </i>
-    <i>
-      <x v="108"/>
-    </i>
-    <i>
-      <x v="109"/>
-    </i>
-    <i>
-      <x v="110"/>
-    </i>
-    <i>
-      <x v="111"/>
-    </i>
-    <i>
-      <x v="112"/>
-    </i>
-    <i>
-      <x v="113"/>
-    </i>
-    <i>
-      <x v="114"/>
-    </i>
-    <i>
-      <x v="115"/>
-    </i>
-    <i>
-      <x v="116"/>
-    </i>
-    <i>
-      <x v="117"/>
-    </i>
-    <i>
-      <x v="118"/>
-    </i>
-    <i>
-      <x v="119"/>
-    </i>
-    <i>
-      <x v="120"/>
-    </i>
-    <i>
-      <x v="121"/>
-    </i>
-    <i>
-      <x v="122"/>
-    </i>
-    <i>
-      <x v="123"/>
-    </i>
-    <i>
-      <x v="124"/>
-    </i>
-    <i>
-      <x v="125"/>
-    </i>
-    <i>
-      <x v="126"/>
-    </i>
-    <i>
-      <x v="127"/>
-    </i>
-    <i>
-      <x v="128"/>
-    </i>
-    <i>
-      <x v="129"/>
-    </i>
-    <i>
-      <x v="130"/>
-    </i>
-    <i>
-      <x v="131"/>
-    </i>
-    <i>
-      <x v="132"/>
-    </i>
-    <i>
-      <x v="133"/>
-    </i>
-    <i>
-      <x v="134"/>
-    </i>
-    <i>
-      <x v="135"/>
-    </i>
-    <i>
-      <x v="136"/>
-    </i>
-    <i>
-      <x v="137"/>
-    </i>
-    <i>
-      <x v="138"/>
-    </i>
-    <i>
-      <x v="139"/>
-    </i>
-    <i>
-      <x v="140"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="2">
-    <pageField fld="11" hier="-1"/>
-    <pageField fld="9" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Count of Promotion" fld="11" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{166599A4-10FF-421A-AFB4-AE0C311C3DFB}" name="PivotTable2" cacheId="331" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="C3:D30" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="18">
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
-      <items count="134">
-        <item x="57"/>
-        <item x="116"/>
-        <item x="10"/>
-        <item x="27"/>
-        <item x="88"/>
-        <item x="19"/>
-        <item x="14"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item x="125"/>
-        <item x="128"/>
-        <item x="121"/>
-        <item x="41"/>
-        <item x="80"/>
-        <item x="93"/>
-        <item x="81"/>
-        <item x="111"/>
-        <item x="82"/>
-        <item x="49"/>
-        <item x="48"/>
-        <item x="68"/>
-        <item x="107"/>
-        <item x="83"/>
-        <item x="42"/>
-        <item x="97"/>
-        <item x="5"/>
-        <item x="11"/>
-        <item x="8"/>
-        <item x="35"/>
-        <item x="25"/>
-        <item x="99"/>
-        <item x="32"/>
-        <item x="22"/>
-        <item x="9"/>
-        <item x="13"/>
-        <item x="126"/>
-        <item x="54"/>
-        <item x="28"/>
-        <item x="53"/>
-        <item x="21"/>
-        <item x="84"/>
-        <item x="20"/>
-        <item x="12"/>
-        <item x="1"/>
-        <item x="86"/>
-        <item x="102"/>
-        <item x="127"/>
-        <item x="30"/>
-        <item x="43"/>
-        <item x="85"/>
-        <item x="112"/>
-        <item x="62"/>
-        <item x="50"/>
-        <item x="98"/>
-        <item x="36"/>
-        <item x="106"/>
-        <item x="17"/>
-        <item x="6"/>
-        <item x="122"/>
-        <item x="52"/>
-        <item x="104"/>
-        <item x="3"/>
-        <item x="7"/>
-        <item x="18"/>
-        <item x="26"/>
-        <item x="103"/>
-        <item x="31"/>
-        <item x="89"/>
-        <item x="118"/>
-        <item x="2"/>
-        <item x="16"/>
-        <item x="55"/>
-        <item x="58"/>
-        <item x="114"/>
-        <item x="33"/>
-        <item x="87"/>
-        <item x="113"/>
-        <item x="69"/>
-        <item x="51"/>
-        <item x="59"/>
-        <item x="101"/>
-        <item x="34"/>
-        <item x="109"/>
-        <item x="61"/>
-        <item x="132"/>
-        <item x="56"/>
-        <item x="64"/>
-        <item x="117"/>
-        <item x="63"/>
-        <item x="100"/>
-        <item x="124"/>
-        <item x="108"/>
-        <item x="115"/>
-        <item x="70"/>
-        <item x="71"/>
-        <item x="72"/>
-        <item x="4"/>
-        <item x="15"/>
-        <item x="65"/>
-        <item x="44"/>
-        <item x="119"/>
-        <item x="105"/>
-        <item x="66"/>
-        <item x="120"/>
-        <item x="123"/>
-        <item x="45"/>
-        <item x="129"/>
-        <item x="130"/>
-        <item x="39"/>
-        <item x="73"/>
-        <item x="110"/>
-        <item x="46"/>
-        <item x="94"/>
-        <item x="74"/>
-        <item x="29"/>
-        <item x="75"/>
-        <item x="90"/>
-        <item x="67"/>
-        <item x="76"/>
-        <item x="38"/>
-        <item x="91"/>
-        <item x="37"/>
-        <item x="40"/>
-        <item x="60"/>
-        <item x="95"/>
-        <item x="77"/>
-        <item x="47"/>
-        <item x="78"/>
-        <item x="131"/>
-        <item x="96"/>
-        <item x="92"/>
-        <item x="79"/>
-        <item h="1" x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisPage" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="35">
-        <item x="15"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item x="12"/>
-        <item x="30"/>
-        <item x="13"/>
-        <item x="19"/>
-        <item x="3"/>
-        <item x="28"/>
-        <item x="1"/>
-        <item x="22"/>
-        <item x="31"/>
-        <item x="16"/>
-        <item x="18"/>
-        <item x="24"/>
-        <item x="26"/>
-        <item x="11"/>
-        <item x="14"/>
-        <item x="27"/>
-        <item x="23"/>
-        <item x="8"/>
-        <item x="21"/>
-        <item x="25"/>
-        <item x="17"/>
-        <item x="10"/>
-        <item x="5"/>
-        <item x="32"/>
-        <item x="33"/>
-        <item x="29"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="20"/>
-        <item x="6"/>
-        <item h="1" x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="27">
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="23"/>
-    </i>
-    <i>
-      <x v="27"/>
-    </i>
-    <i>
-      <x v="33"/>
-    </i>
-    <i>
-      <x v="42"/>
-    </i>
-    <i>
-      <x v="47"/>
-    </i>
-    <i>
-      <x v="49"/>
-    </i>
-    <i>
-      <x v="56"/>
-    </i>
-    <i>
-      <x v="61"/>
-    </i>
-    <i>
-      <x v="69"/>
-    </i>
-    <i>
-      <x v="70"/>
-    </i>
-    <i>
-      <x v="72"/>
-    </i>
-    <i>
-      <x v="74"/>
-    </i>
-    <i>
-      <x v="86"/>
-    </i>
-    <i>
-      <x v="94"/>
-    </i>
-    <i>
-      <x v="96"/>
-    </i>
-    <i>
-      <x v="101"/>
-    </i>
-    <i>
-      <x v="104"/>
-    </i>
-    <i>
-      <x v="108"/>
-    </i>
-    <i>
-      <x v="112"/>
-    </i>
-    <i>
-      <x v="119"/>
-    </i>
-    <i>
-      <x v="120"/>
-    </i>
-    <i>
-      <x v="121"/>
-    </i>
-    <i>
-      <x v="122"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="1">
-    <pageField fld="14" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Count of Recognition (Award" fld="14" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FC177463-ECB6-493F-84C5-BD2B6B5E3667}" name="PivotTable1" cacheId="331" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FC177463-ECB6-493F-84C5-BD2B6B5E3667}" name="PivotTable1" cacheId="472" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:B35" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="18">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -29344,6 +29042,311 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{166599A4-10FF-421A-AFB4-AE0C311C3DFB}" name="PivotTable2" cacheId="472" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="C3:D30" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="18">
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="134">
+        <item x="57"/>
+        <item x="116"/>
+        <item x="10"/>
+        <item x="27"/>
+        <item x="88"/>
+        <item x="19"/>
+        <item x="14"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="125"/>
+        <item x="128"/>
+        <item x="121"/>
+        <item x="41"/>
+        <item x="80"/>
+        <item x="93"/>
+        <item x="81"/>
+        <item x="111"/>
+        <item x="82"/>
+        <item x="49"/>
+        <item x="48"/>
+        <item x="68"/>
+        <item x="107"/>
+        <item x="83"/>
+        <item x="42"/>
+        <item x="97"/>
+        <item x="5"/>
+        <item x="11"/>
+        <item x="8"/>
+        <item x="35"/>
+        <item x="25"/>
+        <item x="99"/>
+        <item x="32"/>
+        <item x="22"/>
+        <item x="9"/>
+        <item x="13"/>
+        <item x="126"/>
+        <item x="54"/>
+        <item x="28"/>
+        <item x="53"/>
+        <item x="21"/>
+        <item x="84"/>
+        <item x="20"/>
+        <item x="12"/>
+        <item x="1"/>
+        <item x="86"/>
+        <item x="102"/>
+        <item x="127"/>
+        <item x="30"/>
+        <item x="43"/>
+        <item x="85"/>
+        <item x="112"/>
+        <item x="62"/>
+        <item x="50"/>
+        <item x="98"/>
+        <item x="36"/>
+        <item x="106"/>
+        <item x="17"/>
+        <item x="6"/>
+        <item x="122"/>
+        <item x="52"/>
+        <item x="104"/>
+        <item x="3"/>
+        <item x="7"/>
+        <item x="18"/>
+        <item x="26"/>
+        <item x="103"/>
+        <item x="31"/>
+        <item x="89"/>
+        <item x="118"/>
+        <item x="2"/>
+        <item x="16"/>
+        <item x="55"/>
+        <item x="58"/>
+        <item x="114"/>
+        <item x="33"/>
+        <item x="87"/>
+        <item x="113"/>
+        <item x="69"/>
+        <item x="51"/>
+        <item x="59"/>
+        <item x="101"/>
+        <item x="34"/>
+        <item x="109"/>
+        <item x="61"/>
+        <item x="132"/>
+        <item x="56"/>
+        <item x="64"/>
+        <item x="117"/>
+        <item x="63"/>
+        <item x="100"/>
+        <item x="124"/>
+        <item x="108"/>
+        <item x="115"/>
+        <item x="70"/>
+        <item x="71"/>
+        <item x="72"/>
+        <item x="4"/>
+        <item x="15"/>
+        <item x="65"/>
+        <item x="44"/>
+        <item x="119"/>
+        <item x="105"/>
+        <item x="66"/>
+        <item x="120"/>
+        <item x="123"/>
+        <item x="45"/>
+        <item x="129"/>
+        <item x="130"/>
+        <item x="39"/>
+        <item x="73"/>
+        <item x="110"/>
+        <item x="46"/>
+        <item x="94"/>
+        <item x="74"/>
+        <item x="29"/>
+        <item x="75"/>
+        <item x="90"/>
+        <item x="67"/>
+        <item x="76"/>
+        <item x="38"/>
+        <item x="91"/>
+        <item x="37"/>
+        <item x="40"/>
+        <item x="60"/>
+        <item x="95"/>
+        <item x="77"/>
+        <item x="47"/>
+        <item x="78"/>
+        <item x="131"/>
+        <item x="96"/>
+        <item x="92"/>
+        <item x="79"/>
+        <item h="1" x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisPage" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="35">
+        <item x="15"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="12"/>
+        <item x="30"/>
+        <item x="13"/>
+        <item x="19"/>
+        <item x="3"/>
+        <item x="28"/>
+        <item x="1"/>
+        <item x="22"/>
+        <item x="31"/>
+        <item x="16"/>
+        <item x="18"/>
+        <item x="24"/>
+        <item x="26"/>
+        <item x="11"/>
+        <item x="14"/>
+        <item x="27"/>
+        <item x="23"/>
+        <item x="8"/>
+        <item x="21"/>
+        <item x="25"/>
+        <item x="17"/>
+        <item x="10"/>
+        <item x="5"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="29"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="20"/>
+        <item x="6"/>
+        <item h="1" x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="27">
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="23"/>
+    </i>
+    <i>
+      <x v="27"/>
+    </i>
+    <i>
+      <x v="33"/>
+    </i>
+    <i>
+      <x v="42"/>
+    </i>
+    <i>
+      <x v="47"/>
+    </i>
+    <i>
+      <x v="49"/>
+    </i>
+    <i>
+      <x v="56"/>
+    </i>
+    <i>
+      <x v="61"/>
+    </i>
+    <i>
+      <x v="69"/>
+    </i>
+    <i>
+      <x v="70"/>
+    </i>
+    <i>
+      <x v="72"/>
+    </i>
+    <i>
+      <x v="74"/>
+    </i>
+    <i>
+      <x v="86"/>
+    </i>
+    <i>
+      <x v="94"/>
+    </i>
+    <i>
+      <x v="96"/>
+    </i>
+    <i>
+      <x v="101"/>
+    </i>
+    <i>
+      <x v="104"/>
+    </i>
+    <i>
+      <x v="108"/>
+    </i>
+    <i>
+      <x v="112"/>
+    </i>
+    <i>
+      <x v="119"/>
+    </i>
+    <i>
+      <x v="120"/>
+    </i>
+    <i>
+      <x v="121"/>
+    </i>
+    <i>
+      <x v="122"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="14" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Count of Recognition (Award" fld="14" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -29635,7 +29638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U366"/>
+  <dimension ref="A1:U367"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15.95" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5.140625" style="1" customWidth="1"/>
@@ -44845,44 +44848,87 @@
       <c r="A366" s="37">
         <v>369</v>
       </c>
-      <c r="B366" s="14" t="s">
+      <c r="B366" s="21" t="s">
         <v>791</v>
       </c>
-      <c r="C366" s="14" t="s">
+      <c r="C366" s="21" t="s">
         <v>549</v>
       </c>
-      <c r="D366" s="14" t="s">
+      <c r="D366" s="21" t="s">
         <v>550</v>
       </c>
-      <c r="E366" s="14" t="s">
+      <c r="E366" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="F366" s="14" t="s">
+      <c r="F366" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="G366" s="14">
+      <c r="G366" s="21">
         <v>8</v>
       </c>
-      <c r="H366" s="14" t="s">
+      <c r="H366" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="I366" s="14" t="s">
+      <c r="I366" s="21" t="s">
         <v>451</v>
       </c>
-      <c r="J366" s="14">
+      <c r="J366" s="21">
         <v>2026</v>
       </c>
-      <c r="K366" s="16"/>
-      <c r="L366" s="16"/>
-      <c r="M366" s="16"/>
-      <c r="N366" s="16"/>
-      <c r="O366" s="16"/>
-      <c r="P366" s="14" t="s">
+      <c r="K366" s="23"/>
+      <c r="L366" s="23"/>
+      <c r="M366" s="23"/>
+      <c r="N366" s="23"/>
+      <c r="O366" s="23"/>
+      <c r="P366" s="21" t="s">
         <v>797</v>
       </c>
-      <c r="Q366" s="16"/>
-      <c r="R366" s="16"/>
+      <c r="Q366" s="23"/>
+      <c r="R366" s="23"/>
       <c r="S366" s="17"/>
+    </row>
+    <row r="367" spans="1:21" ht="15.95" customHeight="1">
+      <c r="A367" s="21">
+        <v>370</v>
+      </c>
+      <c r="B367" s="21" t="s">
+        <v>791</v>
+      </c>
+      <c r="C367" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D367" s="15" t="s">
+        <v>247</v>
+      </c>
+      <c r="E367" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F367" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="G367" s="14">
+        <v>5</v>
+      </c>
+      <c r="H367" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="I367" s="14" t="s">
+        <v>465</v>
+      </c>
+      <c r="J367" s="14">
+        <v>2026</v>
+      </c>
+      <c r="K367" s="16"/>
+      <c r="L367" s="16"/>
+      <c r="M367" s="16"/>
+      <c r="N367" s="16" t="s">
+        <v>798</v>
+      </c>
+      <c r="O367" s="16"/>
+      <c r="P367" s="16"/>
+      <c r="Q367" s="16"/>
+      <c r="R367" s="16"/>
+      <c r="S367" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:T366" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
@@ -44921,12 +44967,12 @@
         <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="13" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>4</v>
@@ -44943,7 +44989,7 @@
         <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -44987,7 +45033,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="B8">
         <v>2</v>
@@ -44998,7 +45044,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="B9">
         <v>114</v>
@@ -45015,7 +45061,7 @@
         <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -45034,7 +45080,7 @@
         <v>36</v>
       </c>
       <c r="H17" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -45048,7 +45094,7 @@
         <v>28</v>
       </c>
       <c r="E18" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="F18" t="s">
         <v>57</v>
@@ -45059,7 +45105,7 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="B19">
         <v>1</v>
@@ -45219,13 +45265,13 @@
         <v>13</v>
       </c>
       <c r="B1" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D1" s="13" t="s">
         <v>11</v>
       </c>
       <c r="E1" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -45233,13 +45279,13 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="D2" s="13" t="s">
         <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -45247,7 +45293,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="C4">
         <f>COUNTA(A4:A93)</f>
@@ -45257,7 +45303,7 @@
         <v>2</v>
       </c>
       <c r="E4" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -46804,10 +46850,10 @@
     </row>
     <row r="137" spans="1:5">
       <c r="A137" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="D137" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
     </row>
     <row r="138" spans="1:5">
@@ -46900,13 +46946,13 @@
     </row>
     <row r="146" spans="1:5">
       <c r="A146" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="B146">
         <v>162</v>
       </c>
       <c r="D146" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="E146">
         <v>91</v>
@@ -46929,7 +46975,7 @@
   <sheetData>
     <row r="2" spans="2:2">
       <c r="B2" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
     </row>
   </sheetData>
@@ -46999,13 +47045,13 @@
         <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>14</v>
       </c>
       <c r="D1" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -47013,13 +47059,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="C3" s="13" t="s">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -47394,7 +47440,7 @@
         <v>2</v>
       </c>
       <c r="C30" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="D30">
         <v>32</v>
@@ -47434,7 +47480,7 @@
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="B35">
         <v>47</v>

</xml_diff>